<commit_message>
points pas tâches unitaire + ajustement des tâches par user stories + burndown chart
</commit_message>
<xml_diff>
--- a/Burndown_Chart_Global_Sprints.xlsx
+++ b/Burndown_Chart_Global_Sprints.xlsx
@@ -462,10 +462,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D2" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3">
@@ -480,7 +480,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>28.33333333333333</v>
+        <v>29.27777777777778</v>
       </c>
       <c r="D3" t="inlineStr"/>
     </row>
@@ -496,7 +496,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>26.66666666666667</v>
+        <v>27.55555555555556</v>
       </c>
       <c r="D4" t="inlineStr"/>
     </row>
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>25</v>
+        <v>25.83333333333333</v>
       </c>
       <c r="D5" t="inlineStr"/>
     </row>
@@ -528,7 +528,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>23.33333333333333</v>
+        <v>24.11111111111111</v>
       </c>
       <c r="D6" t="inlineStr"/>
     </row>
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>21.66666666666666</v>
+        <v>22.38888888888889</v>
       </c>
       <c r="D7" t="inlineStr"/>
     </row>
@@ -560,7 +560,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>20</v>
+        <v>20.66666666666666</v>
       </c>
       <c r="D8" t="inlineStr"/>
     </row>
@@ -576,7 +576,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>18.33333333333333</v>
+        <v>18.94444444444444</v>
       </c>
       <c r="D9" t="inlineStr"/>
     </row>
@@ -592,7 +592,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>16.66666666666666</v>
+        <v>17.22222222222222</v>
       </c>
       <c r="D10" t="inlineStr"/>
     </row>
@@ -608,7 +608,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>15</v>
+        <v>15.5</v>
       </c>
       <c r="D11" t="inlineStr"/>
     </row>
@@ -624,7 +624,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>13.33333333333333</v>
+        <v>13.77777777777778</v>
       </c>
       <c r="D12" t="inlineStr"/>
     </row>
@@ -640,7 +640,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>11.66666666666666</v>
+        <v>12.05555555555555</v>
       </c>
       <c r="D13" t="inlineStr"/>
     </row>
@@ -656,7 +656,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>10</v>
+        <v>10.33333333333333</v>
       </c>
       <c r="D14" t="inlineStr"/>
     </row>
@@ -672,7 +672,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>8.333333333333332</v>
+        <v>8.611111111111111</v>
       </c>
       <c r="D15" t="inlineStr"/>
     </row>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>6.666666666666664</v>
+        <v>6.888888888888886</v>
       </c>
       <c r="D16" t="inlineStr"/>
     </row>
@@ -704,7 +704,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>5</v>
+        <v>5.166666666666664</v>
       </c>
       <c r="D17" t="inlineStr"/>
     </row>
@@ -720,7 +720,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>3.333333333333332</v>
+        <v>3.444444444444443</v>
       </c>
       <c r="D18" t="inlineStr"/>
     </row>
@@ -736,7 +736,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1.666666666666664</v>
+        <v>1.722222222222221</v>
       </c>
       <c r="D19" t="inlineStr"/>
     </row>
@@ -768,10 +768,10 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="D21" t="n">
-        <v>60</v>
+        <v>72</v>
       </c>
     </row>
     <row r="22">
@@ -786,7 +786,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>55.38461538461539</v>
+        <v>66.46153846153847</v>
       </c>
       <c r="D22" t="inlineStr"/>
     </row>
@@ -802,7 +802,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>50.76923076923077</v>
+        <v>60.92307692307692</v>
       </c>
       <c r="D23" t="inlineStr"/>
     </row>
@@ -818,7 +818,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>46.15384615384615</v>
+        <v>55.38461538461539</v>
       </c>
       <c r="D24" t="inlineStr"/>
     </row>
@@ -834,7 +834,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>41.53846153846154</v>
+        <v>49.84615384615385</v>
       </c>
       <c r="D25" t="inlineStr"/>
     </row>
@@ -850,7 +850,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>36.92307692307693</v>
+        <v>44.30769230769231</v>
       </c>
       <c r="D26" t="inlineStr"/>
     </row>
@@ -866,7 +866,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>32.30769230769231</v>
+        <v>38.76923076923077</v>
       </c>
       <c r="D27" t="inlineStr"/>
     </row>
@@ -882,7 +882,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>27.69230769230769</v>
+        <v>33.23076923076923</v>
       </c>
       <c r="D28" t="inlineStr"/>
     </row>
@@ -898,7 +898,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>23.07692307692308</v>
+        <v>27.69230769230769</v>
       </c>
       <c r="D29" t="inlineStr"/>
     </row>
@@ -914,7 +914,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>18.46153846153847</v>
+        <v>22.15384615384615</v>
       </c>
       <c r="D30" t="inlineStr"/>
     </row>
@@ -930,7 +930,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>13.84615384615385</v>
+        <v>16.61538461538461</v>
       </c>
       <c r="D31" t="inlineStr"/>
     </row>
@@ -946,7 +946,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>9.230769230769234</v>
+        <v>11.07692307692308</v>
       </c>
       <c r="D32" t="inlineStr"/>
     </row>
@@ -962,7 +962,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>4.61538461538462</v>
+        <v>5.538461538461547</v>
       </c>
       <c r="D33" t="inlineStr"/>
     </row>
@@ -994,10 +994,10 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D35" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
     <row r="36">
@@ -1012,7 +1012,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>37.5</v>
+        <v>40.83333333333334</v>
       </c>
       <c r="D36" t="inlineStr"/>
     </row>
@@ -1028,7 +1028,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>30</v>
+        <v>32.66666666666667</v>
       </c>
       <c r="D37" t="inlineStr"/>
     </row>
@@ -1044,7 +1044,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>22.5</v>
+        <v>24.5</v>
       </c>
       <c r="D38" t="inlineStr"/>
     </row>
@@ -1060,7 +1060,7 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>15</v>
+        <v>16.33333333333334</v>
       </c>
       <c r="D39" t="inlineStr"/>
     </row>
@@ -1076,7 +1076,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>7.5</v>
+        <v>8.166666666666671</v>
       </c>
       <c r="D40" t="inlineStr"/>
     </row>

</xml_diff>